<commit_message>
EthFw: 11.0.0: Update release notes and collaterals
- Update release notes, datasheet, test reports and
  static analysis reports for SDK 11.00
- Update documentation for default VLAN IDs to
  reflect review comment left on merged PR #620
  on EthFw.

Fixes: ETHFW-2837
Signed-off-by: Siddharth S <s-s9@ti.com>
</commit_message>
<xml_diff>
--- a/docs/traceability_report/ethfw_Traceability_Report.xlsx
+++ b/docs/traceability_report/ethfw_Traceability_Report.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Table of Contents" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Script Input Parameters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Coverage Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Forward Traceability" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Backward Traceability" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Traceability Deviations" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Template Revision History" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table of Contents" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Script Input Parameters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward Traceability" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backward Traceability" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Deviations" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Revision History" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Coverage Summary'!$A$1:$E$3</definedName>
-    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Forward Traceability'!$A$1:$F$4</definedName>
-    <definedName hidden="1" localSheetId="4" name="_xlnm._FilterDatabase">'Backward Traceability'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Coverage Summary'!$A$1:$E$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Forward Traceability'!$A$1:$F$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Backward Traceability'!$A$1:$F$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -77,39 +77,39 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="2" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="3" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -473,9 +473,9 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="10"/>
-    <col customWidth="1" max="2" min="2" width="35"/>
-    <col customWidth="1" max="3" min="3" width="80"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,7 +490,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Copyright (C) 2024 Texas Instruments Incorporated</t>
+          <t>Copyright (C) 2025 Texas Instruments Incorporated</t>
         </is>
       </c>
       <c r="B2" s="5" t="n"/>
@@ -625,10 +625,10 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -641,9 +641,9 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="20"/>
-    <col customWidth="1" max="2" min="2" width="20"/>
-    <col customWidth="1" max="3" min="3" width="35"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -666,7 +666,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2900</t>
+          <t>ETHFW-3041</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -676,12 +676,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2024-11-26 07:22:00.299041-06:00 CDT</t>
+          <t>2025-02-18 03:22:26.036870-06:00 CDT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -694,10 +694,10 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="60"/>
-    <col customWidth="1" max="2" min="2" width="22"/>
-    <col customWidth="1" max="4" min="4" width="60"/>
-    <col customWidth="1" max="5" min="5" width="22"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -771,7 +771,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E3"/>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -781,14 +781,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="20"/>
-    <col customWidth="1" max="2" min="2" width="20"/>
-    <col customWidth="1" max="4" min="4" width="20"/>
-    <col customWidth="1" max="5" min="5" width="20"/>
-    <col customWidth="1" max="6" min="6" width="20"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -822,78 +822,422 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>JACINTOREQ-2621</t>
+          <t>JACINTOREQ-7796</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1199</t>
+          <t>ETHFW-3007,ETHFW-3008,ETHFW-3009</t>
         </is>
       </c>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-1199</t>
+          <t>ETHFW-3007</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2908</t>
+          <t>ETHFW-3032</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Validation</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>JACINTOREQ-554</t>
+          <t>JACINTOREQ-6571</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1199</t>
+          <t>ETHFW-2213,ETHFW-2208</t>
         </is>
       </c>
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-2718</t>
+          <t>ETHFW-2213</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2917,ETHFW-2913,ETHFW-2914,ETHFW-2915,ETHFW-2916</t>
+          <t>ETHFW-3030</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Validation,Validation,Validation,Validation,Validation</t>
+          <t>Validation</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>JACINTOREQ-4908</t>
+          <t>JACINTOREQ-6575</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2718</t>
+          <t>ETHFW-2204,ETHFW-2207,ETHFW-2206</t>
         </is>
       </c>
       <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2204</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3030</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6570</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2201,ETHFW-2202,ETHFW-2211,ETHFW-2199,ETHFW-2203</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2201</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3030</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6623</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2459,ETHFW-2724</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2459</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3038</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-7921</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3010,ETHFW-3011</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2208</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3030</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-7662</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2723</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3010</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3035</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3008</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3031</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3011</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3036</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2207</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3030</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2724</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3039</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2206</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3030</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2202</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3030</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2211</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3030</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2199</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3037</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2203</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3030</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3009</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3033</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2723</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-3040</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <autoFilter ref="A1:F19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -903,14 +1247,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="20"/>
-    <col customWidth="1" max="2" min="2" width="20"/>
-    <col customWidth="1" max="4" min="4" width="20"/>
-    <col customWidth="1" max="5" min="5" width="20"/>
-    <col customWidth="1" max="6" min="6" width="20"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -944,46 +1288,46 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-1199</t>
+          <t>ETHFW-3007</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>JACINTOREQ-2621,JACINTOREQ-554</t>
+          <t>JACINTOREQ-7796</t>
         </is>
       </c>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-2908</t>
+          <t>ETHFW-3030</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1199</t>
+          <t>ETHFW-2206,ETHFW-2213,ETHFW-2202,ETHFW-2204,ETHFW-2203,ETHFW-2211,ETHFW-2208,ETHFW-2207,ETHFW-2201</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-2718</t>
+          <t>ETHFW-2213</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>JACINTOREQ-4908</t>
+          <t>JACINTOREQ-6571</t>
         </is>
       </c>
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-2913</t>
+          <t>ETHFW-3031</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -993,17 +1337,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2718</t>
+          <t>ETHFW-3008</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2204</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6575</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-2914</t>
+          <t>ETHFW-3032</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1013,17 +1365,25 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2718</t>
+          <t>ETHFW-3007</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2201</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6570</t>
+        </is>
+      </c>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-2915</t>
+          <t>ETHFW-3033</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1033,17 +1393,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2718</t>
+          <t>ETHFW-3009</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2459</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6623</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-2916</t>
+          <t>ETHFW-3035</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1053,17 +1421,25 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2718</t>
+          <t>ETHFW-3010</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2208</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6571</t>
+        </is>
+      </c>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>ETHFW-2917</t>
+          <t>ETHFW-3036</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1073,13 +1449,253 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2718</t>
-        </is>
-      </c>
+          <t>ETHFW-3011</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3010</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-7921</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3037</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2199</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3008</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-7796</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3038</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2459</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3011</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-7921</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3039</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2724</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2207</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6575</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3040</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2723</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2724</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6623</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2206</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6575</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2202</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6570</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2211</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6570</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2199</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6570</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2203</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-6570</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-3009</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-7796</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>ETHFW-2723</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>JACINTOREQ-7662</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F7"/>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <autoFilter ref="A1:F19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1092,9 +1708,9 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="60"/>
-    <col customWidth="1" max="2" min="2" width="20"/>
-    <col customWidth="1" max="3" min="3" width="80"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1120,7 +1736,7 @@
       <c r="C2" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1133,10 +1749,10 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="20"/>
-    <col customWidth="1" max="2" min="2" width="20"/>
-    <col customWidth="1" max="3" min="3" width="20"/>
-    <col customWidth="1" max="4" min="4" width="20"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1184,6 +1800,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>